<commit_message>
Ischaemic heart disease update
</commit_message>
<xml_diff>
--- a/codelists/ischaemic_heart_disease_raw.xlsx
+++ b/codelists/ischaemic_heart_disease_raw.xlsx
@@ -6074,7 +6074,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>299800012</t>
+          <t>299804015</t>
         </is>
       </c>
       <c r="B118" s="1" t="n">
@@ -6082,12 +6082,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>G34y</t>
+          <t>G34yz</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>G34y.00</t>
+          <t>G34yz00</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Other specified chronic ischaemic heart disease</t>
+          <t>Other specified chronic ischaemic heart disease NOS</t>
         </is>
       </c>
       <c r="H118" s="1" t="n">
@@ -6125,7 +6125,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>299804015</t>
+          <t>299800012</t>
         </is>
       </c>
       <c r="B119" s="1" t="n">
@@ -6133,12 +6133,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>G34yz</t>
+          <t>G34y</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>G34yz00</t>
+          <t>G34y.00</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Other specified chronic ischaemic heart disease NOS</t>
+          <t>Other specified chronic ischaemic heart disease</t>
         </is>
       </c>
       <c r="H119" s="1" t="n">

</xml_diff>

<commit_message>
Ischaemic heart disease final
</commit_message>
<xml_diff>
--- a/codelists/ischaemic_heart_disease_raw.xlsx
+++ b/codelists/ischaemic_heart_disease_raw.xlsx
@@ -6319,7 +6319,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>299804015</t>
+          <t>299800012</t>
         </is>
       </c>
       <c r="B123" s="1" t="n">
@@ -6327,12 +6327,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>G34yz</t>
+          <t>G34y</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>G34yz00</t>
+          <t>G34y.00</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6347,7 +6347,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Other specified chronic ischaemic heart disease NOS</t>
+          <t>Other specified chronic ischaemic heart disease</t>
         </is>
       </c>
       <c r="H123" s="1" t="n">
@@ -6370,7 +6370,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>299800012</t>
+          <t>299804015</t>
         </is>
       </c>
       <c r="B124" s="1" t="n">
@@ -6378,12 +6378,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>G34y</t>
+          <t>G34yz</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>G34y.00</t>
+          <t>G34yz00</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6398,7 +6398,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Other specified chronic ischaemic heart disease</t>
+          <t>Other specified chronic ischaemic heart disease NOS</t>
         </is>
       </c>
       <c r="H124" s="1" t="n">
@@ -6656,7 +6656,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>6860251000006115</t>
+          <t>299750014</t>
         </is>
       </c>
       <c r="B130" s="1" t="n">
@@ -6664,10 +6664,14 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>^ESCTIS686025</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr"/>
+          <t>G31yz</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>G31yz00</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>414545008</t>
@@ -6680,7 +6684,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Ischemic heart disease</t>
+          <t>Other acute and subacute ischaemic heart disease NOS</t>
         </is>
       </c>
       <c r="H130" s="1" t="n">
@@ -6703,7 +6707,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>299750014</t>
+          <t>6860251000006115</t>
         </is>
       </c>
       <c r="B131" s="1" t="n">
@@ -6711,14 +6715,10 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>G31yz</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>G31yz00</t>
-        </is>
-      </c>
+          <t>^ESCTIS686025</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
           <t>414545008</t>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Other acute and subacute ischaemic heart disease NOS</t>
+          <t>Ischemic heart disease</t>
         </is>
       </c>
       <c r="H131" s="1" t="n">

</xml_diff>